<commit_message>
fix: resolve excel header parsing issue in OrderView
</commit_message>
<xml_diff>
--- a/sample data/확장주문검색_20260709100921_36166302.xls.xlsx
+++ b/sample data/확장주문검색_20260709100921_36166302.xls.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\damon\Desktop\ANTIGRAVITY\wyshboard\sample data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83DE0D35-B4C2-4010-BC0A-152CCEC5CBD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1E9F911-ED8B-4C37-842F-245E5C01DE75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{905BE1A5-70CD-4FEA-904D-52588A30771A}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1478" uniqueCount="457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1478" uniqueCount="458">
   <si>
     <t>관리번호</t>
   </si>
@@ -1394,6 +1394,10 @@
   </si>
   <si>
     <t>010-8938-1587</t>
+  </si>
+  <si>
+    <t>위시크림 블랙카카오밀키웨이</t>
+    <phoneticPr fontId="21" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -2427,6 +2431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6C8F92B-7015-4DD9-8269-1131934B0D6D}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:BG60"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3844,7 +3849,7 @@
       </c>
       <c r="BG9" s="2"/>
     </row>
-    <row r="10" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:59" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>984305</v>
       </c>
@@ -3886,7 +3891,7 @@
       </c>
       <c r="P10" s="2"/>
       <c r="Q10" s="3" t="s">
-        <v>69</v>
+        <v>457</v>
       </c>
       <c r="R10" s="2"/>
       <c r="S10" s="2"/>
@@ -9283,7 +9288,7 @@
       </c>
       <c r="BG46" s="2"/>
     </row>
-    <row r="47" spans="1:59" ht="27" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:59" ht="27" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="3">
         <v>984095</v>
       </c>
@@ -9325,7 +9330,7 @@
       </c>
       <c r="P47" s="2"/>
       <c r="Q47" s="3" t="s">
-        <v>139</v>
+        <v>457</v>
       </c>
       <c r="R47" s="2"/>
       <c r="S47" s="2"/>
@@ -9430,7 +9435,7 @@
       </c>
       <c r="BG47" s="2"/>
     </row>
-    <row r="48" spans="1:59" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:59" ht="40.5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="3">
         <v>984094</v>
       </c>
@@ -9577,7 +9582,7 @@
       </c>
       <c r="BG48" s="2"/>
     </row>
-    <row r="49" spans="1:59" ht="27" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:59" ht="27" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="3">
         <v>984092</v>
       </c>
@@ -9724,7 +9729,7 @@
       </c>
       <c r="BG49" s="2"/>
     </row>
-    <row r="50" spans="1:59" ht="27" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:59" ht="27" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="3">
         <v>984091</v>
       </c>
@@ -9871,7 +9876,7 @@
       </c>
       <c r="BG50" s="2"/>
     </row>
-    <row r="51" spans="1:59" ht="27" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:59" ht="27" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="3">
         <v>984090</v>
       </c>
@@ -10018,7 +10023,7 @@
       </c>
       <c r="BG51" s="2"/>
     </row>
-    <row r="52" spans="1:59" ht="27" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:59" ht="27" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="3">
         <v>984089</v>
       </c>
@@ -10165,7 +10170,7 @@
       </c>
       <c r="BG52" s="2"/>
     </row>
-    <row r="53" spans="1:59" ht="27" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:59" ht="27" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="3">
         <v>984088</v>
       </c>
@@ -10312,7 +10317,7 @@
       </c>
       <c r="BG53" s="2"/>
     </row>
-    <row r="54" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:59" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="3">
         <v>984087</v>
       </c>
@@ -10459,7 +10464,7 @@
       </c>
       <c r="BG54" s="2"/>
     </row>
-    <row r="55" spans="1:59" ht="27" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:59" ht="27" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="3">
         <v>984086</v>
       </c>
@@ -10606,7 +10611,7 @@
       </c>
       <c r="BG55" s="2"/>
     </row>
-    <row r="56" spans="1:59" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:59" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="3">
         <v>984085</v>
       </c>
@@ -10753,7 +10758,7 @@
       </c>
       <c r="BG56" s="2"/>
     </row>
-    <row r="57" spans="1:59" ht="27" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:59" ht="27" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="3">
         <v>984084</v>
       </c>
@@ -10900,7 +10905,7 @@
       </c>
       <c r="BG57" s="2"/>
     </row>
-    <row r="58" spans="1:59" ht="27" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:59" ht="27" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="3">
         <v>984083</v>
       </c>
@@ -11047,7 +11052,7 @@
       </c>
       <c r="BG58" s="2"/>
     </row>
-    <row r="59" spans="1:59" ht="27" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:59" ht="27" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="3">
         <v>984082</v>
       </c>
@@ -11194,7 +11199,7 @@
       </c>
       <c r="BG59" s="2"/>
     </row>
-    <row r="60" spans="1:59" ht="27" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:59" ht="27" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="3">
         <v>984081</v>
       </c>
@@ -11342,7 +11347,13 @@
       <c r="BG60" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BG60" xr:uid="{E6C8F92B-7015-4DD9-8269-1131934B0D6D}"/>
+  <autoFilter ref="A1:BG60" xr:uid="{E6C8F92B-7015-4DD9-8269-1131934B0D6D}">
+    <filterColumn colId="14">
+      <filters>
+        <filter val="위시그릭 019"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="21" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>